<commit_message>
getting critical shear stress using tau=rho g R s
</commit_message>
<xml_diff>
--- a/antecedent_conditions/field_data/results/tauc_estimates_with_equations.xlsx
+++ b/antecedent_conditions/field_data/results/tauc_estimates_with_equations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\shear_stress_paper\antecedent_conditions\field_data\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41AA45B-660A-4BDA-9A73-32CC1F99843B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50EAE043-8BDA-4627-93CA-E02D3423CB6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="1104" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Interpolated Rising" sheetId="1" r:id="rId1"/>

</xml_diff>